<commit_message>
More changes to the GUI to making it more autonomous. Next is to get the actual tracker working to get it running roughly then I can add nice final touches.
</commit_message>
<xml_diff>
--- a/souls_death_workout.xlsx
+++ b/souls_death_workout.xlsx
@@ -1,57 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mjbel\Documents\Projects\CS_Proj\soulsDeath2pushUps\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{06971334-E3B8-4DD2-96F5-EEA6F22707E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{B3C7315A-DFBB-4BE5-8032-4EEFCA1886D5}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -70,21 +46,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -404,10 +439,75 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31323046-232F-41F0-8A11-FAA17A0C4BDF}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Death Number</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Death Number</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Death Number</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Death Number</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Death Number</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Roughly did all of excel_manager and some other small details
</commit_message>
<xml_diff>
--- a/souls_death_workout.xlsx
+++ b/souls_death_workout.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mjbel\Documents\Projects\CS_Proj\soulsDeath2pushUps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA1F02F1-5484-452D-9BE6-80DA84726314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{143B8018-DA78-412F-A29B-5E19FDCBDEAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17340" yWindow="2340" windowWidth="16605" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RAW DATA" sheetId="1" r:id="rId1"/>
@@ -21,12 +21,24 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
-  <si>
-    <t>GAME</t>
-  </si>
-  <si>
-    <t>DEATHS</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+  <si>
+    <t>Elden Ring</t>
+  </si>
+  <si>
+    <t>Dark Souls III</t>
+  </si>
+  <si>
+    <t>Dark Souls II</t>
+  </si>
+  <si>
+    <t>Dark Souls</t>
+  </si>
+  <si>
+    <t>Sekiro</t>
+  </si>
+  <si>
+    <t>Demon's Souls</t>
   </si>
 </sst>
 </file>
@@ -398,15 +410,40 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Did a lot... game_monitoring for looking for a game start, and added a lot more to main, then more touches to every other class
</commit_message>
<xml_diff>
--- a/souls_death_workout.xlsx
+++ b/souls_death_workout.xlsx
@@ -8,20 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mjbel\Documents\Projects\CS_Proj\soulsDeath2pushUps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{143B8018-DA78-412F-A29B-5E19FDCBDEAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD6690A6-4FA9-479B-9B27-386C39203D18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17340" yWindow="2340" windowWidth="16605" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10695" yWindow="2340" windowWidth="23250" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="RAW DATA" sheetId="1" r:id="rId1"/>
-    <sheet name="ORGANIZED DATA" sheetId="2" r:id="rId2"/>
+    <sheet name="input" sheetId="1" r:id="rId1"/>
+    <sheet name="output" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Elden Ring</t>
   </si>
@@ -39,6 +39,51 @@
   </si>
   <si>
     <t>Demon's Souls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nightreign </t>
+  </si>
+  <si>
+    <t>Total Deaths:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Pushups: </t>
+  </si>
+  <si>
+    <t>Elden Ring:</t>
+  </si>
+  <si>
+    <t>Nightreign:</t>
+  </si>
+  <si>
+    <t>Dark Souls III:</t>
+  </si>
+  <si>
+    <t>Dark Souls II:</t>
+  </si>
+  <si>
+    <t>Dark Souls:</t>
+  </si>
+  <si>
+    <t>Sekiro:</t>
+  </si>
+  <si>
+    <t>Demon's Souls:</t>
+  </si>
+  <si>
+    <t>Past Data</t>
+  </si>
+  <si>
+    <t>Debt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pushups Needed: </t>
+  </si>
+  <si>
+    <t>Totals</t>
+  </si>
+  <si>
+    <t>Workout Entry</t>
   </si>
 </sst>
 </file>
@@ -410,40 +455,48 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -453,9 +506,71 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2939F13A-6FA1-4006-9A07-3CA5585E6089}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>